<commit_message>
kant deont + debates
</commit_message>
<xml_diff>
--- a/DigSite/New Arcaism/uarm 2026 a/maestría/Grupos Formulación de investigación.xlsx
+++ b/DigSite/New Arcaism/uarm 2026 a/maestría/Grupos Formulación de investigación.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitData\ArchaeologyJourney\DigSite\New Arcaism\uarm 2026 a\maestría\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70598F39-688A-4384-8B3F-B0D71B315608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ACD3C27-103B-4939-A622-4A7BE45FE745}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="615" yWindow="150" windowWidth="11925" windowHeight="10920" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="615" yWindow="0" windowWidth="17325" windowHeight="10920" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lista" sheetId="2" state="hidden" r:id="rId1"/>
@@ -880,7 +880,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -902,6 +902,7 @@
     <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1368,7 +1369,7 @@
       <c r="E8" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="F8" s="20" t="s">
+      <c r="F8" s="21" t="s">
         <v>150</v>
       </c>
     </row>
@@ -1388,7 +1389,7 @@
       <c r="E9" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="21"/>
+      <c r="F9" s="22"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10">
@@ -1406,7 +1407,7 @@
       <c r="E10" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="F10" s="21"/>
+      <c r="F10" s="22"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="10">
@@ -1424,7 +1425,7 @@
       <c r="E11" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="21"/>
+      <c r="F11" s="22"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="10">
@@ -1442,7 +1443,7 @@
       <c r="E12" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="F12" s="21"/>
+      <c r="F12" s="22"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="10">
@@ -1460,7 +1461,7 @@
       <c r="E13" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="F13" s="21"/>
+      <c r="F13" s="22"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="10">
@@ -1478,7 +1479,7 @@
       <c r="E14" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="F14" s="21"/>
+      <c r="F14" s="22"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="10">
@@ -1496,7 +1497,7 @@
       <c r="E15" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="F15" s="22"/>
+      <c r="F15" s="23"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
@@ -1514,7 +1515,7 @@
       <c r="E16" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="F16" s="20" t="s">
+      <c r="F16" s="21" t="s">
         <v>151</v>
       </c>
     </row>
@@ -1534,7 +1535,7 @@
       <c r="E17" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="F17" s="23"/>
+      <c r="F17" s="24"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
@@ -1552,7 +1553,7 @@
       <c r="E18" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="F18" s="23"/>
+      <c r="F18" s="24"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
@@ -1570,7 +1571,7 @@
       <c r="E19" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="F19" s="24"/>
+      <c r="F19" s="25"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="10">
@@ -1588,7 +1589,7 @@
       <c r="E20" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="F20" s="20" t="s">
+      <c r="F20" s="21" t="s">
         <v>152</v>
       </c>
     </row>
@@ -1608,7 +1609,7 @@
       <c r="E21" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="F21" s="23"/>
+      <c r="F21" s="24"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="10">
@@ -1626,7 +1627,7 @@
       <c r="E22" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="F22" s="23"/>
+      <c r="F22" s="24"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="10">
@@ -1644,7 +1645,7 @@
       <c r="E23" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="F23" s="24"/>
+      <c r="F23" s="25"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="2">
@@ -1662,7 +1663,7 @@
       <c r="E24" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="F24" s="25" t="s">
+      <c r="F24" s="26" t="s">
         <v>153</v>
       </c>
     </row>
@@ -1682,7 +1683,7 @@
       <c r="E25" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="F25" s="26"/>
+      <c r="F25" s="27"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
@@ -1700,7 +1701,7 @@
       <c r="E26" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="F26" s="26"/>
+      <c r="F26" s="27"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
@@ -1718,7 +1719,7 @@
       <c r="E27" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="F27" s="26"/>
+      <c r="F27" s="27"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
@@ -1736,7 +1737,7 @@
       <c r="E28" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="F28" s="26"/>
+      <c r="F28" s="27"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="2">
@@ -1754,7 +1755,7 @@
       <c r="E29" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="F29" s="26"/>
+      <c r="F29" s="27"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="2">
@@ -1772,7 +1773,7 @@
       <c r="E30" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="F30" s="26"/>
+      <c r="F30" s="27"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="2">
@@ -1790,7 +1791,7 @@
       <c r="E31" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="F31" s="26"/>
+      <c r="F31" s="27"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="10">
@@ -1808,7 +1809,7 @@
       <c r="E32" s="11" t="s">
         <v>111</v>
       </c>
-      <c r="F32" s="25" t="s">
+      <c r="F32" s="26" t="s">
         <v>154</v>
       </c>
     </row>
@@ -1828,7 +1829,7 @@
       <c r="E33" s="11" t="s">
         <v>115</v>
       </c>
-      <c r="F33" s="26"/>
+      <c r="F33" s="27"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="10">
@@ -1846,7 +1847,7 @@
       <c r="E34" s="11" t="s">
         <v>119</v>
       </c>
-      <c r="F34" s="26"/>
+      <c r="F34" s="27"/>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="10">
@@ -1864,7 +1865,7 @@
       <c r="E35" s="13" t="s">
         <v>122</v>
       </c>
-      <c r="F35" s="26"/>
+      <c r="F35" s="27"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="2">
@@ -1882,7 +1883,7 @@
       <c r="E36" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="F36" s="17" t="s">
+      <c r="F36" s="18" t="s">
         <v>155</v>
       </c>
     </row>
@@ -1890,7 +1891,7 @@
       <c r="A37" s="2">
         <v>30</v>
       </c>
-      <c r="B37" s="7" t="s">
+      <c r="B37" s="17" t="s">
         <v>126</v>
       </c>
       <c r="C37" s="7" t="s">
@@ -1902,7 +1903,7 @@
       <c r="E37" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="F37" s="18"/>
+      <c r="F37" s="19"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="2">
@@ -1920,13 +1921,13 @@
       <c r="E38" s="7" t="s">
         <v>133</v>
       </c>
-      <c r="F38" s="18"/>
+      <c r="F38" s="19"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="2">
         <v>32</v>
       </c>
-      <c r="B39" s="7" t="s">
+      <c r="B39" s="17" t="s">
         <v>134</v>
       </c>
       <c r="C39" s="7" t="s">
@@ -1938,13 +1939,13 @@
       <c r="E39" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="F39" s="18"/>
+      <c r="F39" s="19"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="2">
         <v>33</v>
       </c>
-      <c r="B40" s="7" t="s">
+      <c r="B40" s="17" t="s">
         <v>138</v>
       </c>
       <c r="C40" s="7" t="s">
@@ -1956,7 +1957,7 @@
       <c r="E40" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="F40" s="19"/>
+      <c r="F40" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>